<commit_message>
Fix duplicate Excel sheet crash and ship v1.3.1 export improvements.
Prevent save failures when truncated sheet names collide, refactor workbook export with partial presets and styling, and add inline-edit and semester-start persistence fixes.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/sample/Timetable.xlsx
+++ b/sample/Timetable.xlsx
@@ -31,28 +31,38 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+  <numFmts count="0"/>
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
+      <sz val="11"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill patternType="none">
+        <bgColor/>
+      </patternFill>
     </fill>
     <fill>
-      <patternFill patternType="gray125"/>
+      <patternFill patternType="gray125">
+        <bgColor/>
+      </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left/>
       <right/>
@@ -61,13 +71,15 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -400,166 +412,166 @@
   <dimension ref="A1:M4"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
+      <c r="A1" s="2" t="str">
         <v>ID</v>
       </c>
-      <c r="B1" t="str">
+      <c r="B1" s="2" t="str">
         <v>Module code</v>
       </c>
-      <c r="C1" t="str">
+      <c r="C1" s="2" t="str">
         <v>Module name</v>
       </c>
-      <c r="D1" t="str">
+      <c r="D1" s="2" t="str">
         <v>Activity</v>
       </c>
-      <c r="E1" t="str">
+      <c r="E1" s="2" t="str">
         <v>Type</v>
       </c>
-      <c r="F1" t="str">
+      <c r="F1" s="2" t="str">
         <v>Weekday</v>
       </c>
-      <c r="G1" t="str">
+      <c r="G1" s="2" t="str">
         <v>Start time</v>
       </c>
-      <c r="H1" t="str">
+      <c r="H1" s="2" t="str">
         <v>End time</v>
       </c>
-      <c r="I1" t="str">
+      <c r="I1" s="2" t="str">
         <v>Room</v>
       </c>
-      <c r="J1" t="str">
+      <c r="J1" s="2" t="str">
         <v>Campus</v>
       </c>
-      <c r="K1" t="str">
+      <c r="K1" s="2" t="str">
         <v>Staff</v>
       </c>
-      <c r="L1" t="str">
+      <c r="L1" s="2" t="str">
         <v>Student Groups</v>
       </c>
-      <c r="M1" t="str">
+      <c r="M1" s="2" t="str">
         <v>Size</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" t="str">
+      <c r="B2" s="2" t="str">
         <v>COM769</v>
       </c>
-      <c r="C2" t="str">
+      <c r="C2" s="2" t="str">
         <v>Example Module A</v>
       </c>
-      <c r="D2" t="str">
+      <c r="D2" s="2" t="str">
         <v>COM769 LEC GRP A</v>
       </c>
-      <c r="E2" t="str">
+      <c r="E2" s="2" t="str">
         <v>Lecture</v>
       </c>
-      <c r="F2" t="str">
+      <c r="F2" s="2" t="str">
         <v>Wednesday</v>
       </c>
-      <c r="G2" t="str">
+      <c r="G2" s="2" t="str">
         <v>09:30</v>
       </c>
-      <c r="H2" t="str">
+      <c r="H2" s="2" t="str">
         <v>11:30</v>
       </c>
-      <c r="I2" t="str">
+      <c r="I2" s="2" t="str">
         <v/>
       </c>
-      <c r="J2" t="str">
+      <c r="J2" s="2" t="str">
         <v>London RAV</v>
       </c>
-      <c r="K2" t="str">
+      <c r="K2" s="2" t="str">
         <v>Tutor Name</v>
       </c>
-      <c r="L2" t="str">
+      <c r="L2" s="2" t="str">
         <v>Grp A</v>
       </c>
-      <c r="M2">
+      <c r="M2" s="2">
         <v>10</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3">
+      <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="B3" t="str">
+      <c r="B3" s="2" t="str">
         <v>COM769</v>
       </c>
-      <c r="C3" t="str">
+      <c r="C3" s="2" t="str">
         <v>Example Module A</v>
       </c>
-      <c r="D3" t="str">
+      <c r="D3" s="2" t="str">
         <v>COM769 SEM GRP A</v>
       </c>
-      <c r="E3" t="str">
+      <c r="E3" s="2" t="str">
         <v>Seminar</v>
       </c>
-      <c r="F3" t="str">
+      <c r="F3" s="2" t="str">
         <v>Friday</v>
       </c>
-      <c r="G3" t="str">
+      <c r="G3" s="2" t="str">
         <v>09:30</v>
       </c>
-      <c r="H3" t="str">
+      <c r="H3" s="2" t="str">
         <v>11:30</v>
       </c>
-      <c r="I3" t="str">
+      <c r="I3" s="2" t="str">
         <v/>
       </c>
-      <c r="J3" t="str">
+      <c r="J3" s="2" t="str">
         <v>London RAV</v>
       </c>
-      <c r="K3" t="str">
+      <c r="K3" s="2" t="str">
         <v>Tutor Name</v>
       </c>
-      <c r="L3" t="str">
+      <c r="L3" s="2" t="str">
         <v>Grp A</v>
       </c>
-      <c r="M3">
+      <c r="M3" s="2">
         <v>10</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4">
+      <c r="A4" s="2">
         <v>3</v>
       </c>
-      <c r="B4" t="str">
+      <c r="B4" s="2" t="str">
         <v>COM745</v>
       </c>
-      <c r="C4" t="str">
+      <c r="C4" s="2" t="str">
         <v>Example Module B</v>
       </c>
-      <c r="D4" t="str">
+      <c r="D4" s="2" t="str">
         <v>COM745 SEM GRP A</v>
       </c>
-      <c r="E4" t="str">
+      <c r="E4" s="2" t="str">
         <v>Seminar</v>
       </c>
-      <c r="F4" t="str">
+      <c r="F4" s="2" t="str">
         <v>Monday</v>
       </c>
-      <c r="G4" t="str">
+      <c r="G4" s="2" t="str">
         <v>14:30</v>
       </c>
-      <c r="H4" t="str">
+      <c r="H4" s="2" t="str">
         <v>16:30</v>
       </c>
-      <c r="I4" t="str">
+      <c r="I4" s="2" t="str">
         <v/>
       </c>
-      <c r="J4" t="str">
+      <c r="J4" s="2" t="str">
         <v>Birmingham LRH</v>
       </c>
-      <c r="K4" t="str">
+      <c r="K4" s="2" t="str">
         <v>Another Tutor</v>
       </c>
-      <c r="L4" t="str">
+      <c r="L4" s="2" t="str">
         <v>Grp A</v>
       </c>
-      <c r="M4">
+      <c r="M4" s="2">
         <v>8</v>
       </c>
     </row>

</xml_diff>